<commit_message>
feat(productos): Guía Restaurante Gastronómico v2.0 — 18 xlsx (representante de la familia de guías): 0 plantillas sin fórmulas (antes 4), 1.883 fórmulas, plan financiero con proyección real a 3 años (rampa de arranque = cash flow), escandallo con raciones/merma/IVA, menu engineering Kasavana & Smith completo, brigada 40 h con registro de jornada y SMI 2026, checklists legal/sanitario vigentes con 390 ítems, calculadora CAPEX coherente con la necesidad, 41/41 hojas protegidas; docx/PDF pendientes de T7
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017kK9BRAxpAsfsxudgwH42U
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/guia-restaurante-gastronomico/calculadora-capex.xlsx
+++ b/astro-site/public/dl/guia-restaurante-gastronomico/calculadora-capex.xlsx
@@ -22,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.00 €"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -69,8 +69,22 @@
       <color rgb="001565C0"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001565C0"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -87,6 +101,16 @@
       <patternFill patternType="solid">
         <fgColor rgb="002D2D2D"/>
         <bgColor rgb="002D2D2D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F5E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002D2D2D"/>
       </patternFill>
     </fill>
   </fills>
@@ -116,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -144,6 +168,39 @@
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -510,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -561,7 +618,7 @@
     </row>
     <row r="8"/>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>Celdas verdes = campos editables</t>
         </is>
@@ -569,13 +626,48 @@
     </row>
     <row r="10"/>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Versión 1.1 · agosto 2026 · aichef.pro/guia-restaurante-gastronomico · info@aichef.pro</t>
+      <c r="A11" s="13" t="n"/>
+    </row>
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>Esta calculadora es la hoja de RANGOS DE MERCADO. TU CAPEX, el que va al banco, se rellena en plan-financiero-3-anos.xlsx, hoja «Inversión», que trae la correspondencia concepto → categoría de esta hoja. Los dos libros se comparan; ninguno lee del otro (un .xlsx movido de carpeta daría #REF!).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>Los rangos cubren la NECESIDAD TOTAL, no solo la obra y el equipo: incluyen la preapertura (rentas y nóminas antes de abrir) y el fondo de maniobra de seis meses, que son las dos partidas que hunden a quien abre. Las dos llegan con la cifra del plan financiero de este kit como EJEMPLO en la columna verde; ajústalas a tu caso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16"/>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>Para editar la estructura o una celda que no esté en verde: Revisar → Desproteger hoja (no tiene contraseña).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>Diseñado por John Guerrero — chef y consultor gastronómico desde 2010, en cocina desde los 17 años · johnguerrero.es</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>Versión 2.0 · agosto 2026 · aichef.pro/guia-restaurante-gastronomico · info@aichef.pro</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
   <mergeCells count="2">
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A1:C1"/>
@@ -599,15 +691,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="47" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="52" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -656,9 +749,14 @@
           <t>Tu Presupuesto (€)</t>
         </is>
       </c>
+      <c r="G4" s="15" t="inlineStr">
+        <is>
+          <t>De dónde sale este rango</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="n">
+      <c r="A5" s="16" t="n">
         <v>1</v>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -675,10 +773,10 @@
       <c r="E5" s="9" t="n">
         <v>450000</v>
       </c>
-      <c r="F5" s="10" t="n"/>
+      <c r="F5" s="17" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="n">
+      <c r="A6" s="16" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="8" t="inlineStr">
@@ -690,20 +788,25 @@
         <v>55000</v>
       </c>
       <c r="D6" s="9" t="n">
-        <v>90000</v>
+        <v>110000</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>150000</v>
-      </c>
-      <c r="F6" s="10" t="n"/>
+        <v>180000</v>
+      </c>
+      <c r="F6" s="17" t="n"/>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>El rango alto llega a 180.000 € porque el checklist-equipamiento-cocina.xlsx de este mismo pack tasa 161.430,40 € para una cocina completa con Josper, horno mixto de 10 GN, abatidor y dos cámaras.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="n">
+      <c r="A7" s="16" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Mobiliario sala (65 plazas)</t>
+          <t>Mobiliario sala (65 plazas)</t>
         </is>
       </c>
       <c r="C7" s="9" t="n">
@@ -715,10 +818,10 @@
       <c r="E7" s="9" t="n">
         <v>120000</v>
       </c>
-      <c r="F7" s="10" t="n"/>
+      <c r="F7" s="17" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="n">
+      <c r="A8" s="16" t="n">
         <v>4</v>
       </c>
       <c r="B8" s="8" t="inlineStr">
@@ -735,10 +838,10 @@
       <c r="E8" s="9" t="n">
         <v>65000</v>
       </c>
-      <c r="F8" s="10" t="n"/>
+      <c r="F8" s="17" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n">
+      <c r="A9" s="16" t="n">
         <v>5</v>
       </c>
       <c r="B9" s="8" t="inlineStr">
@@ -755,10 +858,10 @@
       <c r="E9" s="9" t="n">
         <v>100000</v>
       </c>
-      <c r="F9" s="10" t="n"/>
+      <c r="F9" s="17" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="n">
+      <c r="A10" s="16" t="n">
         <v>6</v>
       </c>
       <c r="B10" s="8" t="inlineStr">
@@ -775,10 +878,10 @@
       <c r="E10" s="9" t="n">
         <v>80000</v>
       </c>
-      <c r="F10" s="10" t="n"/>
+      <c r="F10" s="17" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="n">
+      <c r="A11" s="16" t="n">
         <v>7</v>
       </c>
       <c r="B11" s="8" t="inlineStr">
@@ -795,10 +898,10 @@
       <c r="E11" s="9" t="n">
         <v>25000</v>
       </c>
-      <c r="F11" s="10" t="n"/>
+      <c r="F11" s="17" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="n">
+      <c r="A12" s="16" t="n">
         <v>8</v>
       </c>
       <c r="B12" s="8" t="inlineStr">
@@ -815,10 +918,10 @@
       <c r="E12" s="9" t="n">
         <v>20000</v>
       </c>
-      <c r="F12" s="10" t="n"/>
+      <c r="F12" s="17" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="n">
+      <c r="A13" s="16" t="n">
         <v>9</v>
       </c>
       <c r="B13" s="8" t="inlineStr">
@@ -835,10 +938,10 @@
       <c r="E13" s="9" t="n">
         <v>30000</v>
       </c>
-      <c r="F13" s="10" t="n"/>
+      <c r="F13" s="17" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="n">
+      <c r="A14" s="16" t="n">
         <v>10</v>
       </c>
       <c r="B14" s="8" t="inlineStr">
@@ -855,30 +958,37 @@
       <c r="E14" s="9" t="n">
         <v>20000</v>
       </c>
-      <c r="F14" s="10" t="n"/>
+      <c r="F14" s="17" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="n">
+      <c r="A15" s="16" t="n">
         <v>11</v>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>Fondo de maniobra (6 meses)</t>
+          <t>Fondo de maniobra (6 meses)</t>
         </is>
       </c>
       <c r="C15" s="9" t="n">
-        <v>60000</v>
+        <v>180000</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>120000</v>
+        <v>450000</v>
       </c>
       <c r="E15" s="9" t="n">
-        <v>200000</v>
-      </c>
-      <c r="F15" s="10" t="n"/>
+        <v>950000</v>
+      </c>
+      <c r="F15" s="19" t="n">
+        <v>934320.48</v>
+      </c>
+      <c r="G15" s="18" t="inlineStr">
+        <is>
+          <t>Estos tres números son un rango de mercado; el TUYO lo calcula plan-financiero-3-anos.xlsx, hoja «Inversión», con TUS costes fijos. Seis meses del escenario realista de este pack son 6 × 155.720,08 € = 934.320,48 €, que es la cifra de ejemplo de la columna verde y la que marca el rango alto. Ajústala a tu caso.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="n">
+      <c r="A16" s="16" t="n">
         <v>12</v>
       </c>
       <c r="B16" s="8" t="inlineStr">
@@ -895,36 +1005,91 @@
       <c r="E16" s="9" t="n">
         <v>15000</v>
       </c>
-      <c r="F16" s="10" t="n"/>
+      <c r="F16" s="17" t="n"/>
     </row>
     <row r="17">
+      <c r="A17" s="20" t="n">
+        <v>13</v>
+      </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
+          <t>Preapertura (rentas y nóminas antes de abrir)</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="n">
+        <v>40000</v>
+      </c>
+      <c r="D17" s="12" t="n">
+        <v>110000</v>
+      </c>
+      <c r="E17" s="12" t="n">
+        <v>250000</v>
+      </c>
+      <c r="F17" s="21" t="n">
+        <v>221603.36</v>
+      </c>
+      <c r="G17" s="18" t="inlineStr">
+        <is>
+          <t>Rentas y suministros del local antes de abrir (la licencia tarda 4‑8 meses) más las nóminas de la brigada durante la formación. La cifra verde, 221.603,36 €, es la de ejemplo del plan financiero de este kit (6 meses de renta + 2 de nómina); ajústala a tu caso. Sin esta fila, la calculadora pedía menos dinero del que el propio plan dice que hace falta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="11" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C17" s="12">
-        <f>SUM(C5:C16)</f>
-        <v>373000.0</v>
-      </c>
-      <c r="D17" s="12">
-        <f>SUM(D5:D16)</f>
-        <v>703000.0</v>
-      </c>
-      <c r="E17" s="12">
-        <f>SUM(E5:E16)</f>
-        <v>1275000.0</v>
-      </c>
-      <c r="F17" s="12">
-        <f>SUM(F5:F16)</f>
-        <v>0.0</v>
-      </c>
+      <c r="C18" s="22">
+        <f>SUM(C5:C17)</f>
+        <v>533000.0</v>
+      </c>
+      <c r="D18" s="22">
+        <f>SUM(D5:D17)</f>
+        <v>1163000.0</v>
+      </c>
+      <c r="E18" s="22">
+        <f>SUM(E5:E17)</f>
+        <v>2305000.0</v>
+      </c>
+      <c r="F18" s="22">
+        <f>IF(COUNT(F5:F17)=0,"",SUM(F5:F17))</f>
+        <v>1155923.8399999999</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="C19" s="23" t="n"/>
+      <c r="D19" s="23" t="n"/>
+      <c r="E19" s="23" t="n"/>
+      <c r="F19" s="23" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Tu presupuesto frente al rango de mercado</t>
+        </is>
+      </c>
+      <c r="B20" s="23" t="n"/>
+      <c r="C20" s="23" t="n"/>
+      <c r="D20" s="23" t="n"/>
+      <c r="E20" s="23" t="n"/>
+      <c r="F20" t="str">
+        <f>IF(COUNT(F5:F17)=0,"",IF(COUNT(F5:F17)&lt;COUNTIF($B$5:$B$17,"&lt;&gt;"),"Columna incompleta: el TOTAL sólo suma las filas que has rellenado",IF(F18&lt;C18,"Por debajo del rango bajo",IF(F18&gt;E18,"Por encima del rango alto","Dentro del rango"))))</f>
+        <v>Columna incompleta: el TOTAL sólo suma las filas que has rellenado</v>
+      </c>
+      <c r="G20" s="23" t="n"/>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
   <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16 F17" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Importe no válido" error="Escribe un número mayor o igual que 0." type="decimal" operator="greaterThanOrEqual">
+      <formula1>0</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>

</xml_diff>